<commit_message>
docs: refresh handoff; record DR-01 PASS and U-* findings in the tracker
DR-01 run headless against production: 10 pages plus a six-step client-side
journey, 0 console errors / uncaught exceptions / 4xx / broken assets. The 81
net::ERR_ABORTED events are Next.js ?_rsc= prefetches to our own host and fire
while the page merely idles, so they are expected behaviour.

Tracker Sheet 1 now carries all 16 issues including the U-* findings that had
only ever been verbal, with fix notes and the measured numbers (/ was 47.2s
cold, now 0.22s; 80 suite-replay rows to 0). BE-A03 flips FAIL -> PASS.

Handoff rewritten: records the Hinglish correction, the corrected local run
commands (port 8000, server/.env auto-loads), and the gotchas learned this
session - gh is absent, the dashboard key is not qa-alpha, and the reusable
puppeteer-core harness.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Loupe_Test_Tracker.xlsx
+++ b/docs/Loupe_Test_Tracker.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -615,10 +615,14 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr"/>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>1d4db2e - decoration-time branch on all four function kinds (plain, generator, async def, async generator); @loupe.span decorator fixed the same way. 11 new tests, all 5 mutations caught. Shipped in loupe-sdk 0.3.2 on 2026-08-20 and verified by installing from PyPI into a clean venv.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -962,7 +966,11 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Re-confirmed on production 2026-09-01: GET /traces/00000000-0000-0000-0000-000000000000 returns HTTP 200, not 404. Still open.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1002,10 +1010,292 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Shipped in 0.3.2 alongside L-001 (dd6686e).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>L-014</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>SDK</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>@loupe.span decorator does not support async generator tools</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>The decorator form handles plain and async def functions. An async generator tool is not supported because the replay freeze/edit path has no defined behaviour for a stream - there is no correct answer to 'how many items should the frozen output yield'.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>sdk/loupe/core.py</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>DR-01 / L-001 work</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>By design</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Documented in the span() docstring; the loupe.span() context manager works for these.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>U-001</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>No landing page; / waited on the backend cold start</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>The app opened straight onto the traces table, which is a server component, so first paint waited for Render's free tier to wake from its ~15 min sleep.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>dashboard/app/page.tsx</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>DR-03</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>5918e34 - static landing page at /, traces list moved to /traces. Measured on production: / was 47.2s on a cold backend, now 0.22s with x-vercel-cache HIT. The page makes zero API calls by design; adding a live stat would turn it dynamic again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>U-002</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>UI is plain - wants motion / imagery / 3D</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Cosmetic. Recommended instead: the landing page (done), an auto-playing demo GIF of the killer flow, and light polish. Showing the product beats decoration.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>dashboard/</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>DR-03</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Landing page shipped; demo GIF slot exists but holds a static mock (Track D).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>U-003</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>/suites returned 404 in production</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>The suites pages existed locally but had never been pushed.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>dashboard/app/suites/</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>DR-03</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Pushed 3e27508. Re-verified 2026-09-01: /suites returns 200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>U-004</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>/suites leads with 'x 0/15 passed', which reads as a broken tool</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>It actually means the run caught 15 regressions - a success for the product. The /suite_runs/[id] page already frames it correctly ('this run would block the PR'); lift that framing up to the list.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>dashboard/app/suites/page.tsx</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>DR-03</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>U-005</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Traces list page 1 buried the interesting runs</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Page 1 was a wall of near-identical rows, pushing the real agent traces onto later pages.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>server/app/routers/traces.py + dashboard/app/traces/page.tsx</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>DR-03</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Partially fixed</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>645df42 - GET /v1/traces gained an is_replay filter and the list defaults to hiding suite replays behind a 'Show replays' toggle. On production this took the '(suite replay)' rows from 80 to 0. REMAINING: page 1 is still 15x genre_extract + 5x triage_repo originals, and all 9 cinerater traces - the actual demo agent - sit on page 2. Needs a separate fix (name filter, or reseed so the interesting traces are newest).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I11"/>
@@ -1199,17 +1489,17 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>output = coroutine repr, duration 0ms, spans lost, raise recorded as success</t>
+          <t>RETESTED 2026-08-19 on the fix: awaited result {'answer': '42'}, duration 51ms, 1 span captured, and a raised ValueError recorded as status=error. Was: coroutine repr, 0ms, 0 spans, status=success.</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>L-001</t>
+          <t>L-001 (fixed, shipped in 0.3.2)</t>
         </is>
       </c>
     </row>
@@ -6850,9 +7140,21 @@
           <t>Zero red errors. Note any warnings</t>
         </is>
       </c>
-      <c r="G83" s="4" t="inlineStr"/>
-      <c r="H83" s="4" t="inlineStr"/>
-      <c r="I83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Automated with headless Chrome (puppeteer-core) against production on 2026-09-01. Swept 10 pages - landing, traces list, replays toggle, status=error, trace detail, branch diff, suites, suite detail, suite run, unknown trace id - then a six-step client-side journey: load /, click through to /traces, toggle replays, open a trace, browser Back, reload. RESULT: 0 console errors, 0 console warnings, 0 uncaught exceptions, 0 HTTP 4xx/5xx, 0 broken assets (35 _next assets checked across 3 pages). The only network events were 81 net::ERR_ABORTED on Next.js prefetch requests (?_rsc=), all to our own host; these also occur while the page merely idles, so they are normal App Router prefetch behaviour, not a defect.</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>Script: scratchpad dr01/dr01b.mjs. Hydration checked by waiting 3s after each step and by an explicit reload step.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6920,9 +7222,21 @@
           <t>Can a stranger tell what Loupe does and why it is impressive? Write down what confused you</t>
         </is>
       </c>
-      <c r="G85" s="4" t="inlineStr"/>
-      <c r="H85" s="4" t="inlineStr"/>
-      <c r="I85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Fresh-eyes recruiter pass. Produced findings U-001 (no landing page + cold-start first paint), U-002 (UI too plain), U-004 (/suites leads with '0/15 passed'), U-005 (traces list page 1 buried the real runs).</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>U-001 and U-003 now fixed; U-005 partially fixed; U-002 and U-004 still open. See Sheet 1.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: record DR-04 results — U-005 closed, L-015/L-016 fixed, U-006 open
DR-04 walked the killer flow on production and found two blockers, both
now fixed: the revoked Groq key still on Render (L-015) and the retired
llama-3.3-70b-versatile that made every stored trace un-replayable
(L-016, ADR B13). U-006 stays open: production has no branchable failed
trace, so the intended "failed run -> fix" demo has no starting point.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Loupe_Test_Tracker.xlsx
+++ b/docs/Loupe_Test_Tracker.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1288,12 +1288,153 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Partially fixed</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>645df42 - GET /v1/traces gained an is_replay filter and the list defaults to hiding suite replays behind a 'Show replays' toggle. On production this took the '(suite replay)' rows from 80 to 0. REMAINING: page 1 is still 15x genre_extract + 5x triage_repo originals, and all 9 cinerater traces - the actual demo agent - sit on page 2. Needs a separate fix (name filter, or reseed so the interesting traces are newest).</t>
+          <t>Part one (2026-08-19): is_replay filter hid 80 suite replays. Part two (2026-09-04, commit 299bff7): GET /v1/traces takes an exact `name` filter applied in SQL (before LIMIT, so has_more stays honest); dashboard shows agent chips All/cinerater/genre_extract/triage_repo, and name is carried through status, the replay toggle and pagination. 7 server tests + a 36-check headless-browser suite; mutation-checked by dropping name from the Next link (3 tests failed). Verified on production: cinerater chip -&gt; 9 rows on page 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>L-015</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Server/Ops</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Production GROQ_API_KEY was revoked - every branch failed with 401</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Found by DR-04 on 2026-09-07. Branching any production trace produced a trace whose error was 'API 401: Invalid API Key'. The key on Render was the one revoked during L-013 and was never replaced. Invisible to every page-level check: HTTP was 200, the console was clean, and the failure lived inside the trace body.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Render env GROQ_API_KEY</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Branched trace error block on production</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>New Groq key set on Render 2026-09-07. The same key backs JudgeService, so suite runs were broken by the same cause. Lesson recorded: a 200 response can carry a failed run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>L-016</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Server/Replay</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Retired provider model made every stored trace un-replayable</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>After L-015 was fixed the branch failed again with 'the model llama-3.3-70b-versatile does not exist'. Groq had retired every Llama chat model. The branch engine re-runs the model recorded on the original span, so the retirement broke replay for all historical traces - not just ours.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>server/app/routers/replays.py</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Branched trace error on production, DR-04</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>ADR B13 + commit 07f59a1. ModelNotFoundError is raised only when the provider says the model itself is gone (matched on the body; providers disagree on 400 vs 404). _invoke_llm retries once on settings.replay_fallback_model (openai/gpt-oss-120b, Groq-served) and records metadata.model_substituted {from,to}; a 'model swapped' badge shows it in the span tree and the diff. A 401 or rate limit is never retried - that would have hidden L-015. judge_backend default moved too. 4 tests, both mutations caught. Verified end-to-end against the real Groq API locally: status error -&gt; success, span model gpt-oss-120b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>U-006</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>No branchable failed trace exists on production - the killer demo cannot be walked</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>DR-04, 2026-09-07. Production has exactly one failed original trace (triage_repo) and it contains a single span. SpanTree offers 'Branch from here' only when something runs after the span (canBranch = started_at &lt; maxStart), so that trace correctly shows 'Nothing runs after this span' instead. The demo in claude.md - failed run, wrong tool call, branch, fix - has no starting point on the live instance.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>production data / dashboard SpanTree</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>DR-04 headless walkthrough</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Needs a seeded failed trace shaped like the intended demo: a wrong tool call followed by further spans. Blocks Track D (killer-demo recording).</t>
         </is>
       </c>
     </row>
@@ -7269,9 +7410,21 @@
           <t>Report every moment you had to think, wait, or explain something</t>
         </is>
       </c>
-      <c r="G86" s="4" t="inlineStr"/>
-      <c r="H86" s="4" t="inlineStr"/>
-      <c r="I86" s="4" t="inlineStr"/>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>Walked on production 2026-09-07 with headless Chrome. Navigation and ergonomics are sound: /traces -&gt; cinerater chip -&gt; trace -&gt; expand span -&gt; 'Branch from here' -&gt; JSON editor prefilled -&gt; Continue -&gt; lands on the branched trace with 'View diff' and 'View original trace'. 0 console errors throughout. The diff renders a status banner, token/cost/latency deltas and per-span pairs. TWO BLOCKERS FOUND: (1) L-015 - every branch failed with 'API 401 Invalid API Key' because Render still held the key revoked during L-013; (2) L-016 - after that fix, 'model llama-3.3-70b-versatile does not exist' because Groq retired every Llama chat model, making all stored traces un-replayable. Both fixed. Also U-006: production has no branchable failed trace, so the intended 'failed run -&gt; fix' demo cannot be walked at all. TIMINGS: first /traces hit 10-12s on a cold Render backend, every later navigation 1-3s, branch submit 2.8s - warm the backend before recording.</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>DONE (2 blockers found, both fixed; U-006 open)</t>
+        </is>
+      </c>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>Script: scratchpad dr01/dr04.mjs and dr04b.mjs (puppeteer-core, system Chrome).</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: record DR-02 PASS — polling stops when nothing is running
Counted requests by path rather than by ?_rsc=: link prefetches carry the
same marker as router.refresh polls, which overstated polling 3x on the
first pass. Production idles at 0 polls on a finished suite run, a
finished trace and the traces list; a 3.6s branch polled exactly once at
the 2500ms interval and then stopped.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Loupe_Test_Tracker.xlsx
+++ b/docs/Loupe_Test_Tracker.xlsx
@@ -7328,9 +7328,21 @@
           <t>Polling stops when nothing is running; no request storm</t>
         </is>
       </c>
-      <c r="G84" s="4" t="inlineStr"/>
-      <c r="H84" s="4" t="inlineStr"/>
-      <c r="I84" s="4" t="inlineStr"/>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Automated with headless Chrome, 2026-09-21. Counted every request the page made to our own host, split by whether it hit the page's OWN path (a router.refresh poll) or another path (a Next.js link prefetch) - both carry ?_rsc=, so counting RSC alone overstates polling 3x. PRODUCTION: finished suite run idle 45s = 0 requests; finished trace idle 45s = 0 polls; /traces list idle 30s = 0 requests. A branched trace page fires 6 RSC on load, all prefetches (/diff, the original trace, /traces) and 0 polls - same category as DR-01's 81 prefetch aborts. LOCAL (exact, to isolate the running state): a branch that ran 3.6s produced exactly 1 poll, matching the 2500ms AutoRefresh interval, then 0 over 30s idle. Polling starts when status is running and stops the moment it is not. No request storm.</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>AutoRefresh is mounted only under a running guard (suite_runs 2000ms, suites 2000ms, trace 2500ms) or inside an in-progress early return (replay/branch diff 3000ms), so the interval is cleared on unmount. Script: scratchpad dr02/dr02*.mjs.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: close U-006 — the killer demo now has a starting point on production
Seeded the failing CineRater run to the live instance and walked the whole
flow in a headless browser: the failed trace shows "Branch from here" on
the wrong parse span, editing 1997 to 2023 branches to success, and the
diff reads "Branch fixed the run: error -> success".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Loupe_Test_Tracker.xlsx
+++ b/docs/Loupe_Test_Tracker.xlsx
@@ -1429,12 +1429,12 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Needs a seeded failed trace shaped like the intended demo: a wrong tool call followed by further spans. Blocks Track D (killer-demo recording).</t>
+          <t>Commit 6c41244 + seeded to production 2026-09-21. examples/cinerater/failing_demo.py is agent.recommend with the empty-result guard removed - the commonest bug in tool-using agents. The catalogue holds 2022-2025 films, so a 1997 query makes the parse LLM emit a year nothing matches, search_movies returns 0 rows, and the unguarded index lookup raises IndexError. Parse runs at temperature 0 so it reproduces. Trace: llm groq.chat -&gt; {genre:Sci-Fi, year:1997}, then tool search_movies -&gt; count 0, status error. Seeded from a neutral directory so the public traceback carries no home path or username. Verified on production with headless Chrome: 'Branch from here' appears on the wrong span, editing 1997 -&gt; 2023 produces a branched trace with status success, and the diff reads 'Branch fixed the run: error -&gt; success'. 0 console errors. Trace ac0276fd-31bf-4e15-89ed-9d5d9120c621. Caveat for the recording: the dry-run ghost shows would_have with the ORIGINAL year, because a server-side branch does not re-run tools - loupe.replay (SDK) is the leg where the edit propagates for real.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: new README screenshots from production, in killer-demo order (DR-05)
The old traces-list and trace-detail shots predated the agent chips and the
landing page, and there was no screenshot of a run being fixed.

Three new shots, dark theme at 2x: the failed CineRater run leading the
list, the span tree with the wrong parse output and "Branch from here", and
the diff reading "Branch fixed the run: error -> success". The README now
walks those three in order and keeps the SDK-replay trio below as the
deeper case where the edit propagates through real tools.

Two problems caught while shooting: a cinerater-filtered list showed empty
Tokens and Cost columns (those seeded runs carry neither), and the first
detail shot was framed mid-page with the failure block off-screen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Loupe_Test_Tracker.xlsx
+++ b/docs/Loupe_Test_Tracker.xlsx
@@ -7469,9 +7469,21 @@
           <t>Screenshot-worthy with no visual embarrassment</t>
         </is>
       </c>
-      <c r="G87" s="4" t="inlineStr"/>
-      <c r="H87" s="4" t="inlineStr"/>
-      <c r="I87" s="4" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>Captured from production 2026-09-21, dark theme, 1440 wide at 2x for retina. Three screens in killer-demo order: the traces list with the failed cinerater run leading, the failed trace with the wrong parse output and 'Branch from here' visible, and the diff reading 'Branch fixed the run: error -&gt; success'. TWO PROBLEMS FOUND AND FIXED WHILE SHOOTING: (1) the first traces-list shot was filtered to cinerater, whose seeded runs carry no token or cost data, so both columns were a column of dashes - the unfiltered list was used instead, because genre_extract rows carry tokens AND cost and the failed run is newest so it still leads. (2) The first trace-detail shot was framed mid-page: the 'This run failed' block was off-screen and the bottom half was the replay form. Reframed by measuring the distance from the failure block to the branch button and sizing the viewport to fit both. Seeded from a neutral directory so no home path or username appears in the public traceback. README rewritten to lead with these three.</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>docs/traces-list.png, docs/trace-detail.png, docs/branch-fixed.png. The older branch-diff-1/2/3 kept below them: they show the SDK-side replay where the edit propagates through real tools, which the server-side branch cannot do. Script: scratchpad dr02/dr05*.mjs.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: record L-017 (spans could not explain an empty answer) and the real-app demo pair
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Loupe_Test_Tracker.xlsx
+++ b/docs/Loupe_Test_Tracker.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1434,7 +1434,54 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Commit 6c41244 + seeded to production 2026-09-21. examples/cinerater/failing_demo.py is agent.recommend with the empty-result guard removed - the commonest bug in tool-using agents. The catalogue holds 2022-2025 films, so a 1997 query makes the parse LLM emit a year nothing matches, search_movies returns 0 rows, and the unguarded index lookup raises IndexError. Parse runs at temperature 0 so it reproduces. Trace: llm groq.chat -&gt; {genre:Sci-Fi, year:1997}, then tool search_movies -&gt; count 0, status error. Seeded from a neutral directory so the public traceback carries no home path or username. Verified on production with headless Chrome: 'Branch from here' appears on the wrong span, editing 1997 -&gt; 2023 produces a branched trace with status success, and the diff reads 'Branch fixed the run: error -&gt; success'. 0 console errors. Trace ac0276fd-31bf-4e15-89ed-9d5d9120c621. Caveat for the recording: the dry-run ghost shows would_have with the ORIGINAL year, because a server-side branch does not re-run tools - loupe.replay (SDK) is the leg where the edit propagates for real.</t>
+          <t>Commit 6c41244 + seeded to production 2026-09-21. examples/cinerater/failing_demo.py is agent.recommend with the empty-result guard removed - the commonest bug in tool-using agents. The catalogue holds 2022-2025 films, so a 1997 query makes the parse LLM emit a year nothing matches, search_movies returns 0 rows, and the unguarded index lookup raises IndexError. Parse runs at temperature 0 so it reproduces. Trace: llm groq.chat -&gt; {genre:Sci-Fi, year:1997}, then tool search_movies -&gt; count 0, status error. Seeded from a neutral directory so the public traceback carries no home path or username. Verified on production with headless Chrome: 'Branch from here' appears on the wrong span, editing 1997 -&gt; 2023 produces a branched trace with status success, and the diff reads 'Branch fixed the run: error -&gt; success'. 0 console errors. Trace ac0276fd-31bf-4e15-89ed-9d5d9120c621. Caveat for the recording: the dry-run ghost shows would_have with the ORIGINAL year, because a server-side branch does not re-run tools - loupe.replay (SDK) is the leg where the edit propagates for real. UPDATE 2026-09-21: production also carries the real CineRater pipeline now - a before/after pair of multi_agent_recommend traces (0e8dbfde shows the silent degradation with the truncation badges, 13d0a0df the fixed run). That pair is a DIAGNOSIS demo, not a branch demo: the ranker's prompt is built by the app's Python from the parsed profile, so a server-side branch of the analyst span would not propagate (the B6 boundary). The toy cinerater trace remains the clickable error -&gt; success branch demo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>L-017</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>SDK</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>LLM spans could not tell an empty answer from a truncated one</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Found by dogfooding Loupe on the real CineRater app. A span whose output is {"content": ""} says the model returned nothing but not why - a refusal, a content filter and a truncation are indistinguishable. The app had moved onto a reasoning model (openai/gpt-oss-120b) keeping its old max_tokens; the hidden reasoning pass is paid from the same budget, so it consumed all of it and the answer came back empty with finish_reason='length'. Nothing raised, logs clean, HTTP 200. Measured: 1885 chars of reasoning and 0 of answer at max_tokens=500; 2523 and 0 at 800.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>sdk/loupe/integrations/*</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Production trace 0e8dbfde on the live demo</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>SDK 0.3.3, commit 02d3011. LLM spans now carry finish_reason, empty_answer and reasoning_chars in metadata for openai, groq and anthropic - only when it is not the boring answer, so normal spans stay clean, and never for a tool-calling turn (one of the tests caught that false positive before it shipped). Anthropic's 'max_tokens' is normalised to 'length'. Reasoning text is never stored, only its length. Dashboard shows a 'truncated' / 'no answer - truncated' badge. 12 tests, mutation-checked. NOT YET PUBLISHED to PyPI.</t>
         </is>
       </c>
     </row>

</xml_diff>